<commit_message>
Update drains_auditing XLSX and primarydrains GeoJSON
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E914D1F5-8EDC-415D-8236-99CDBBFD9DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155DA7C4-75BF-4C13-B1A1-39934B552F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="91">
   <si>
     <t>area</t>
   </si>
@@ -272,6 +272,27 @@
   </si>
   <si>
     <t>234,235,236,237,242,245,248,249,251</t>
+  </si>
+  <si>
+    <t>name_id</t>
+  </si>
+  <si>
+    <t>srujan_k</t>
+  </si>
+  <si>
+    <t>chetan_k</t>
+  </si>
+  <si>
+    <t>amaresh</t>
+  </si>
+  <si>
+    <t>Aditya</t>
+  </si>
+  <si>
+    <t>Banaswadi</t>
+  </si>
+  <si>
+    <t>H400</t>
   </si>
 </sst>
 </file>
@@ -1133,428 +1154,461 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="G3" t="s">
+      <c r="F3" s="1"/>
+      <c r="H3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
       <c r="B5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>20</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
       <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="G6" t="s">
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>26</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="1">
+      <c r="D8" s="1">
         <v>87</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>29</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="G9" t="s">
+      <c r="F9" s="1"/>
+      <c r="H9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="1">
+      <c r="D10" s="1">
         <v>267</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>36</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="E11" s="1" t="s">
+      <c r="D11" s="1"/>
+      <c r="F11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="1">
+      <c r="D12" s="1">
         <v>270</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="G12" t="s">
+      <c r="F12" s="1"/>
+      <c r="H12" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="1">
+      <c r="D13" s="1">
         <v>268</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="G13" t="s">
+      <c r="F13" s="1"/>
+      <c r="H13" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="G14" t="s">
+      <c r="F14" s="1"/>
+      <c r="H14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="G15" t="s">
+      <c r="F15" s="1"/>
+      <c r="H15" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>46</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="G16" t="s">
+      <c r="F16" s="1"/>
+      <c r="H16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="1">
+      <c r="D17" s="1">
         <v>211</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="G17" t="s">
+      <c r="F17" s="1"/>
+      <c r="H17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>52</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>56</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="1"/>
+      <c r="F19" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>57</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>58</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="1">
+      <c r="D20" s="1">
         <v>269</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="G20" t="s">
+      <c r="F20" s="1"/>
+      <c r="H20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>61</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="1">
+      <c r="D21" s="1">
         <v>40</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>64</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E24" s="1"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="1">
+        <v>89</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="H22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Redesign audit_status panel: fixed side panel with team details, map legend overlay
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155DA7C4-75BF-4C13-B1A1-39934B552F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58A1C5B-13B3-4E36-9C74-BE31227B5F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="108">
   <si>
     <t>area</t>
   </si>
@@ -274,18 +274,9 @@
     <t>234,235,236,237,242,245,248,249,251</t>
   </si>
   <si>
-    <t>name_id</t>
-  </si>
-  <si>
     <t>srujan_k</t>
   </si>
   <si>
-    <t>chetan_k</t>
-  </si>
-  <si>
-    <t>amaresh</t>
-  </si>
-  <si>
     <t>Aditya</t>
   </si>
   <si>
@@ -293,6 +284,66 @@
   </si>
   <si>
     <t>H400</t>
+  </si>
+  <si>
+    <t>brb_3</t>
+  </si>
+  <si>
+    <t>brb_2</t>
+  </si>
+  <si>
+    <t>brb_1</t>
+  </si>
+  <si>
+    <t>brb_4</t>
+  </si>
+  <si>
+    <t>mcc</t>
+  </si>
+  <si>
+    <t>rnsit</t>
+  </si>
+  <si>
+    <t>apu_ess</t>
+  </si>
+  <si>
+    <t>anu_g</t>
+  </si>
+  <si>
+    <t>team_captain_name</t>
+  </si>
+  <si>
+    <t>team_crew_name</t>
+  </si>
+  <si>
+    <t>Richa Shreebalaji</t>
+  </si>
+  <si>
+    <t>Aihika Sharma, Divya Puramshetty, Joy Banerjee, Maitrey Deshpande, Anagha V Nanjangud, Taha Mama, Shalini Vailaya, Aveline Thomas, Vijay, Shubhang</t>
+  </si>
+  <si>
+    <t>Mod Foundation &amp; Oorvani Foundation</t>
+  </si>
+  <si>
+    <t>Madhuri Mandava, Divya Puramshetty , Aihika sharma, Richa, Nikhil Nayak , Adith D H, Harinath, Akshat kumar, Jishnu Ravindran, Lakshmi Hegde , Bharat, Angel</t>
+  </si>
+  <si>
+    <t>Aanchal Aggarwal, Aditya Srinivas K, Ajay Singh, Albert Felix, Ashritha, Bharath AL, Debabrata Malik, Deepika Nair, Divya Puramshetty, Druid, Joseph, Kirti, Lakshmi Jagadish, Magarajeswari, Mandanna, Maria Biju, Pradeep, Prashanth AP, Pratham R. Goel, Riya Rahiman, Sakshi Reddy, Sharada Venugopal, Shanmitha Raghu, Shri Vishnu SP, Shreyas Isaac, Shubh, Sireesh Kodali, Soundararajan Rajagopalan, Vinita</t>
+  </si>
+  <si>
+    <t>Aaradhana, Prapulla Chandra D, Aihika Sharma A, Arkachari Pooja, Diksha Jain, Dr Ravindranath C, Gouravi, Govind ShriHari J, Pooja Pawar, Priyanka Salunkhe, Reena Rathi, Samuel Soares, Dr. Sankar Rajkumar, Shanmitha Raghu, Sharada Venugopal, Shreelekha K, Sowmya Muralidhar, Swaminaatha Krishnan, Vani Shetty, Vindhya A H</t>
+  </si>
+  <si>
+    <t>img_id</t>
+  </si>
+  <si>
+    <t>Nikhil Nayak</t>
+  </si>
+  <si>
+    <t>Aadhya Arvind, Abhay Menon, Amrutha Hannah, Cherry Goyal, Prakriti Richa, Smeet, Sruthi Iyer, Trishaa Manda</t>
+  </si>
+  <si>
+    <t>Adith D H, Aishwarya GP, Akanksh Singh, Alankrita Singh, Abhineeth K R, Bhakthi S P, Bhoomika, Dhatri V A, Gayithri, Hrishik Ponnappa, J V Benakasree, Kaustubha K, Manu T, Monish N M, Monishree H, Nihal N, Nikhil Kumar Rao, Prathyush J, Rudra Chakraborty, Shabrinath C, Shamshitha T, Shreyas P H, Shubham Kumar, Sreelekha Vennapusa, Sudhanshu Suman, Tanmay P Shetty, V Koushik, B Varshitha Sri, Vamshi Ganesh B, Varun A, Yashas P</t>
   </si>
 </sst>
 </file>
@@ -776,9 +827,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1154,461 +1208,524 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>84</v>
-      </c>
       <c r="C1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="H3" t="s">
+      <c r="G3" s="1"/>
+      <c r="I3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>20</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="1"/>
-      <c r="H6" t="s">
+      <c r="G6" s="1"/>
+      <c r="I6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>26</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>87</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>29</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="1"/>
-      <c r="H9" t="s">
+      <c r="G9" s="1"/>
+      <c r="I9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>267</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>36</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="F11" s="1" t="s">
+      <c r="E11" s="1"/>
+      <c r="G11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>38</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
       <c r="C12" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="1">
+      <c r="E12" s="1">
         <v>270</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>41</v>
       </c>
-      <c r="F12" s="1"/>
-      <c r="H12" t="s">
+      <c r="G12" s="1"/>
+      <c r="I12" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J12" t="s">
+        <v>100</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
       <c r="C13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="1">
+      <c r="E13" s="1">
         <v>268</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="1"/>
-      <c r="H13" t="s">
+      <c r="G13" s="1"/>
+      <c r="I13" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J13" t="s">
+        <v>100</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="180" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
       <c r="C14" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="1"/>
-      <c r="H14" t="s">
+      <c r="G14" s="1"/>
+      <c r="I14" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J14" t="s">
+        <v>100</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
       <c r="C15" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="1"/>
-      <c r="H15" t="s">
+      <c r="G15" s="1"/>
+      <c r="I15" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J15" t="s">
+        <v>100</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>46</v>
       </c>
       <c r="C16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="H16" t="s">
+      <c r="G16" s="1"/>
+      <c r="I16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="180" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
       <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="1">
+      <c r="E17" s="1">
         <v>211</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="1"/>
-      <c r="H17" t="s">
+      <c r="G17" s="1"/>
+      <c r="I17" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>105</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>52</v>
       </c>
       <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>55</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>56</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J18" t="s">
+        <v>98</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
       <c r="C19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="F19" s="1" t="s">
+      <c r="E19" s="1"/>
+      <c r="G19" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>57</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>58</v>
       </c>
       <c r="C20" t="s">
+        <v>95</v>
+      </c>
+      <c r="D20" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="1">
+      <c r="E20" s="1">
         <v>269</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="1"/>
-      <c r="H20" t="s">
+      <c r="G20" s="1"/>
+      <c r="I20" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>61</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="1">
+      <c r="E21" s="1">
         <v>40</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>63</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>64</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" s="1">
         <v>89</v>
       </c>
-      <c r="C22" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22" s="1">
-        <v>89</v>
-      </c>
-      <c r="E22" t="s">
-        <v>90</v>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="H22" t="s">
+      <c r="F22" t="s">
+        <v>87</v>
+      </c>
+      <c r="G22" s="1"/>
+      <c r="I22" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F24" s="1"/>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add institute field to captain section; guard null DOM refs
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58A1C5B-13B3-4E36-9C74-BE31227B5F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15B5783-5292-421A-8C84-61C9E26E164E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="111">
   <si>
     <t>area</t>
   </si>
@@ -344,13 +344,32 @@
   </si>
   <si>
     <t>Adith D H, Aishwarya GP, Akanksh Singh, Alankrita Singh, Abhineeth K R, Bhakthi S P, Bhoomika, Dhatri V A, Gayithri, Hrishik Ponnappa, J V Benakasree, Kaustubha K, Manu T, Monish N M, Monishree H, Nihal N, Nikhil Kumar Rao, Prathyush J, Rudra Chakraborty, Shabrinath C, Shamshitha T, Shreyas P H, Shubham Kumar, Sreelekha Vennapusa, Sudhanshu Suman, Tanmay P Shetty, V Koushik, B Varshitha Sri, Vamshi Ganesh B, Varun A, Yashas P</t>
+  </si>
+  <si>
+    <t>RNSIT MUN Society</t>
+  </si>
+  <si>
+    <t>Azim Premji University ESS Club</t>
+  </si>
+  <si>
+    <r>
+      <t>team_captain_institute</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -484,6 +503,22 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -827,12 +862,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1208,10 +1245,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1242,8 +1279,11 @@
       <c r="K1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1266,7 +1306,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1283,8 +1323,9 @@
       <c r="I3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1304,7 +1345,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1327,7 +1368,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1345,7 +1386,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1368,7 +1409,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1385,7 +1426,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1403,7 +1444,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1426,7 +1467,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -1441,7 +1482,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -1468,7 +1509,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1495,7 +1536,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="180" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1522,7 +1563,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="135" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1549,7 +1590,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>46</v>
       </c>
@@ -1573,7 +1614,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="180" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="180" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1599,8 +1640,11 @@
       <c r="K17" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="L17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -1631,8 +1675,11 @@
       <c r="K18" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -1656,7 +1703,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>58</v>
       </c>
@@ -1680,7 +1727,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>61</v>
       </c>
@@ -1703,7 +1750,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>86</v>
       </c>
@@ -1721,10 +1768,10 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G24" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update styles and auditing data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15B5783-5292-421A-8C84-61C9E26E164E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DE95F9-E6DB-4CC8-AF12-8A5C54FE3004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -352,24 +352,14 @@
     <t>Azim Premji University ESS Club</t>
   </si>
   <si>
-    <r>
-      <t>team_captain_institute</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Segoe UI"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
+    <t>team_captain_institute</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,16 +499,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9.9"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -862,14 +842,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1279,7 +1258,7 @@
       <c r="K1" t="s">
         <v>97</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update drains_auditing XLSX with institute data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90235E31-F65B-49A6-9C65-E188748EF137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EBDD66-CBE7-4C93-9637-645ED98C62E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -1592,11 +1592,11 @@
       <c r="I16" t="s">
         <v>42</v>
       </c>
+      <c r="J16" t="s">
+        <v>48</v>
+      </c>
       <c r="K16" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="L16" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="180" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Make audit_status responsive and update data
- Add mobile and tablet responsive layout for side panel, map, legend, and search
- Update drains_auditing.xlsx
- Update primarydrains.geojson

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EBDD66-CBE7-4C93-9637-645ED98C62E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2074A034-05A7-49E2-979B-B86B1BD03B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="116">
   <si>
     <t>area</t>
   </si>
@@ -356,6 +356,18 @@
   </si>
   <si>
     <t>Ajay P, Aradhana J, Arjun P, Arshad, Cezanne Ali, Jagadeeswaran B, Jeesta Ghosh, Jenica Angelin, Jeya Shreya S, Malavika, Mayur Jeevan Das, Niharika Bedwal, Prakriti Mukherjee, Prakruti P C, R Swathi, Raghav Kumar, Ria Jagadev, Shradha Mishra, Soumili Santra, Sreeyuktha M V, Sudit Ilin, Tania Noble, Vaishnavi, Vishruti B</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>90,274</t>
+  </si>
+  <si>
+    <t>Aditya S</t>
+  </si>
+  <si>
+    <t>Vivek Matthew</t>
   </si>
 </sst>
 </file>
@@ -1742,19 +1754,40 @@
       <c r="D22" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="1">
-        <v>89</v>
+      <c r="E22" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
       <c r="G22" s="1"/>
       <c r="I22" t="s">
+        <v>42</v>
+      </c>
+      <c r="J22" t="s">
+        <v>114</v>
+      </c>
+      <c r="K22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" t="s">
+        <v>85</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="I23" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G24" s="1"/>

</xml_diff>

<commit_message>
Update script, secondarydrains data, and auditing XLSX
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2074A034-05A7-49E2-979B-B86B1BD03B2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738F664B-827B-44B6-9917-3E6264528C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -367,7 +367,7 @@
     <t>Aditya S</t>
   </si>
   <si>
-    <t>Vivek Matthew</t>
+    <t>Vivek Matthew, Sireesh Kodali</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update audit data, GeoJSON, and scripts for both dashboards
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738F664B-827B-44B6-9917-3E6264528C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE9EA66-5699-400C-8840-11DFF1485DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="120">
   <si>
     <t>area</t>
   </si>
@@ -130,9 +130,6 @@
     <t>K200</t>
   </si>
   <si>
-    <t>K207,K208,K206</t>
-  </si>
-  <si>
     <t>JP Nagar</t>
   </si>
   <si>
@@ -259,9 +256,6 @@
     <t>216,217</t>
   </si>
   <si>
-    <t>231,232,233,393</t>
-  </si>
-  <si>
     <t>238,395,394</t>
   </si>
   <si>
@@ -368,6 +362,24 @@
   </si>
   <si>
     <t>Vivek Matthew, Sireesh Kodali</t>
+  </si>
+  <si>
+    <t>K207,K208</t>
+  </si>
+  <si>
+    <t>K206</t>
+  </si>
+  <si>
+    <t>232,233</t>
+  </si>
+  <si>
+    <t>393,231</t>
+  </si>
+  <si>
+    <t>unknown13</t>
+  </si>
+  <si>
+    <t>122</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1251,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1247,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1268,13 +1280,13 @@
         <v>6</v>
       </c>
       <c r="J1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="K1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1285,13 +1297,13 @@
         <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1308,7 +1320,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -1327,13 +1339,13 @@
         <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>
@@ -1347,13 +1359,13 @@
         <v>18</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F5" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s">
         <v>20</v>
@@ -1370,7 +1382,7 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F6" t="s">
         <v>22</v>
@@ -1388,13 +1400,13 @@
         <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F7" t="s">
         <v>25</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H7" t="s">
         <v>26</v>
@@ -1417,7 +1429,10 @@
         <v>29</v>
       </c>
       <c r="I8" t="s">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="J8" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1428,369 +1443,414 @@
         <v>31</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" t="s">
-        <v>32</v>
+        <v>119</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>118</v>
       </c>
       <c r="G9" s="1"/>
       <c r="I9" t="s">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="J9" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="1">
-        <v>267</v>
+        <v>31</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="H10" t="s">
-        <v>36</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G10" s="1"/>
       <c r="I10" t="s">
         <v>11</v>
       </c>
+      <c r="J10" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
       </c>
       <c r="E11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="H11" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" t="s">
+        <v>41</v>
+      </c>
+      <c r="J11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="1">
+        <v>267</v>
+      </c>
+      <c r="F12" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="G13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" t="s">
+        <v>37</v>
+      </c>
+      <c r="I13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>38</v>
-      </c>
-      <c r="I11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="1">
-        <v>270</v>
-      </c>
-      <c r="F12" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" s="1"/>
-      <c r="I12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J12" t="s">
-        <v>100</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="1">
-        <v>268</v>
-      </c>
-      <c r="F13" t="s">
-        <v>44</v>
-      </c>
-      <c r="G13" s="1"/>
-      <c r="I13" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" t="s">
-        <v>100</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="180" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>45</v>
       </c>
       <c r="C14" t="s">
         <v>89</v>
       </c>
       <c r="D14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="1">
+        <v>270</v>
+      </c>
+      <c r="F14" t="s">
         <v>40</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" t="s">
-        <v>35</v>
       </c>
       <c r="G14" s="1"/>
       <c r="I14" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14" t="s">
+        <v>98</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>42</v>
       </c>
-      <c r="J14" t="s">
-        <v>100</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="135" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>46</v>
-      </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>72</v>
+        <v>39</v>
+      </c>
+      <c r="E15" s="1">
+        <v>268</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G15" s="1"/>
       <c r="I15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="135" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="180" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D16" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="F16" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G16" s="1"/>
       <c r="I16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J16" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="180" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="135" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
-      </c>
-      <c r="E17" s="1">
-        <v>211</v>
+        <v>39</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>71</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G17" s="1"/>
       <c r="I17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="135" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="1"/>
+      <c r="I18" t="s">
+        <v>41</v>
+      </c>
+      <c r="J18" t="s">
+        <v>47</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="180" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="1">
+        <v>211</v>
+      </c>
+      <c r="F19" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" s="1"/>
+      <c r="I19" t="s">
+        <v>41</v>
+      </c>
+      <c r="J19" t="s">
+        <v>103</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="L19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H20" t="s">
+        <v>55</v>
+      </c>
+      <c r="I20" t="s">
+        <v>41</v>
+      </c>
+      <c r="J20" t="s">
+        <v>96</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L20" t="s">
         <v>107</v>
-      </c>
-      <c r="L17" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" t="s">
-        <v>94</v>
-      </c>
-      <c r="D18" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" t="s">
-        <v>55</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H18" t="s">
-        <v>56</v>
-      </c>
-      <c r="I18" t="s">
-        <v>42</v>
-      </c>
-      <c r="J18" t="s">
-        <v>98</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="L18" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" t="s">
-        <v>84</v>
-      </c>
-      <c r="D19" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="G19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H19" t="s">
-        <v>57</v>
-      </c>
-      <c r="I19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J19" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" t="s">
-        <v>59</v>
-      </c>
-      <c r="E20" s="1">
-        <v>269</v>
-      </c>
-      <c r="F20" t="s">
-        <v>60</v>
-      </c>
-      <c r="G20" s="1"/>
-      <c r="I20" t="s">
-        <v>42</v>
-      </c>
-      <c r="J20" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>7</v>
+      </c>
+      <c r="C21" t="s">
+        <v>82</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" s="1">
-        <v>40</v>
-      </c>
-      <c r="F21" t="s">
-        <v>63</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="H21" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="I21" t="s">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="J21" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>86</v>
+        <v>57</v>
+      </c>
+      <c r="C22" t="s">
+        <v>93</v>
       </c>
       <c r="D22" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>112</v>
+        <v>58</v>
+      </c>
+      <c r="E22" s="1">
+        <v>269</v>
       </c>
       <c r="F22" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="G22" s="1"/>
       <c r="I22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J22" t="s">
-        <v>114</v>
-      </c>
-      <c r="K22" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>113</v>
+        <v>61</v>
+      </c>
+      <c r="E23" s="1">
+        <v>40</v>
       </c>
       <c r="F23" t="s">
-        <v>87</v>
-      </c>
-      <c r="G23" s="1"/>
+        <v>62</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H23" t="s">
+        <v>63</v>
+      </c>
       <c r="I23" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F24" t="s">
+        <v>85</v>
+      </c>
       <c r="G24" s="1"/>
+      <c r="I24" t="s">
+        <v>41</v>
+      </c>
+      <c r="J24" t="s">
+        <v>112</v>
+      </c>
+      <c r="K24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>84</v>
+      </c>
+      <c r="D25" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F25" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="1"/>
+      <c r="I25" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G26" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Show team panel for in-progress drains and update audit data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE9EA66-5699-400C-8840-11DFF1485DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA745F6-3436-49E1-98A3-51FE5B766C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
+    <workbookView xWindow="-75" yWindow="105" windowWidth="28980" windowHeight="17280" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
   <sheets>
     <sheet name="drains_auditing" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="127">
   <si>
     <t>area</t>
   </si>
@@ -380,6 +380,27 @@
   </si>
   <si>
     <t>122</t>
+  </si>
+  <si>
+    <t>Suma, Shalini</t>
+  </si>
+  <si>
+    <t>Amarendranath, Prathna, Pranav, Reena, Sheetal, Sireesh, Vivek</t>
+  </si>
+  <si>
+    <t>chetana_rmv</t>
+  </si>
+  <si>
+    <t>ashwin_j</t>
+  </si>
+  <si>
+    <t>poongothai_g</t>
+  </si>
+  <si>
+    <t>Stuti Mehta</t>
+  </si>
+  <si>
+    <t>Joshua, Swarupa, Aruna, Murali</t>
   </si>
 </sst>
 </file>
@@ -1415,10 +1436,13 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
+      <c r="C8" t="s">
+        <v>122</v>
+      </c>
       <c r="D8" t="s">
         <v>28</v>
       </c>
@@ -1433,12 +1457,18 @@
       </c>
       <c r="J8" t="s">
         <v>28</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
       <c r="D9" t="s">
         <v>31</v>
       </c>
@@ -1455,6 +1485,9 @@
       <c r="J9" t="s">
         <v>31</v>
       </c>
+      <c r="K9" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1481,6 +1514,9 @@
       <c r="A11" t="s">
         <v>33</v>
       </c>
+      <c r="C11" t="s">
+        <v>123</v>
+      </c>
       <c r="D11" t="s">
         <v>34</v>
       </c>
@@ -1497,6 +1533,9 @@
       <c r="J11" t="s">
         <v>34</v>
       </c>
+      <c r="K11" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1758,6 +1797,9 @@
       </c>
       <c r="J21" t="s">
         <v>8</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update audit data files
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA745F6-3436-49E1-98A3-51FE5B766C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DA1C56-2AA9-4643-BD16-708DB569F739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-75" yWindow="105" windowWidth="28980" windowHeight="17280" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
   <sheets>
     <sheet name="drains_auditing" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="142">
   <si>
     <t>area</t>
   </si>
@@ -401,6 +401,51 @@
   </si>
   <si>
     <t>Joshua, Swarupa, Aruna, Murali</t>
+  </si>
+  <si>
+    <t>Nandini Layout</t>
+  </si>
+  <si>
+    <t>MSRIT</t>
+  </si>
+  <si>
+    <t>msrit</t>
+  </si>
+  <si>
+    <t>337,335</t>
+  </si>
+  <si>
+    <t>V205,V202</t>
+  </si>
+  <si>
+    <t>Ramaiah Institute of Technology - School of Architecture</t>
+  </si>
+  <si>
+    <t>Aadhya K, Adarsh Anantpur, Aliza Huq, Ameenaa Nasser, Ankush Hejamadi, Ann Aby, Anusha H, Aravind Cheruvat, Aswathi Sivadasan, Bandri Yashwanth, Bharat A Nair, C Monish Raj, Charmaine S Sawian, Chitra S, Dheeraj S N, Dhruvika G, G Veda Rupa Sri, Gayatri Suryadev Guggari, Ismail Mohammed Khaild, Kavya Jaiswal, Khushi Dharpure, Khushi Jagadeesh, Kushaal Bhargav, Lasya U, Lochan V, M Namrata, M S Ananya, Madhura Choudhury, Manish B M, Manpreeth G S, Mohammad Sahil Mehaboob Athani, Muhammed Umair Noor, N C Ankusha, N Madhumitha, Namrata Gouri S Patil, Pratham P</t>
+  </si>
+  <si>
+    <t>Banshankari</t>
+  </si>
+  <si>
+    <t>bmsca</t>
+  </si>
+  <si>
+    <t>BMSCA</t>
+  </si>
+  <si>
+    <t>Aarushi Gowda, Anil Kumar, Charmi D, Chhavi Rai, Deeksha P, Ezrah, Honnu R Gowda, Jinal, Jyothsna C, Kaustubh, Lahari D, Laksh Jain, Madiha Mariyam, Manchala Varshitha, Megh, Nagireddy Almika, Navya Kawatra, Padma Priya M, Rahul C R, Ramyatha, Rashi Bagrecha, Rohith P S, Sahana Athreyas, Shreya Kishore, Smrithi Meghati, Sonia, Spandana Kedarnath, Supreetha R, Tanushree Tapadia, Tejaswini Ramesh, Tia, Ujwal C V, Ujwal K C</t>
+  </si>
+  <si>
+    <t>BMS College Of Architecture</t>
+  </si>
+  <si>
+    <t>275</t>
+  </si>
+  <si>
+    <t>V100</t>
+  </si>
+  <si>
+    <t>V120</t>
   </si>
 </sst>
 </file>
@@ -1272,10 +1317,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L27"/>
+  <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="57.28515625" customWidth="1"/>
+    <col min="11" max="11" width="60" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1359,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1333,7 +1382,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1352,7 +1401,7 @@
       </c>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1372,7 +1421,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1395,7 +1444,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1413,7 +1462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -1436,7 +1485,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1462,7 +1511,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1489,7 +1538,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1510,7 +1559,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1537,7 +1586,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1560,7 +1609,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -1575,7 +1624,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1602,7 +1651,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -1629,7 +1678,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="180" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1656,7 +1705,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="135" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -1683,7 +1732,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="135" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -1710,7 +1759,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="180" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -1740,7 +1789,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -1775,7 +1824,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -1802,7 +1851,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -1826,7 +1875,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -1849,7 +1898,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>84</v>
       </c>
@@ -1873,7 +1922,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>84</v>
       </c>
@@ -1891,8 +1940,69 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="G26" s="1"/>
+    <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26">
+        <v>276</v>
+      </c>
+      <c r="F26" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" t="s">
+        <v>131</v>
+      </c>
+      <c r="I26" t="s">
+        <v>41</v>
+      </c>
+      <c r="J26" t="s">
+        <v>132</v>
+      </c>
+      <c r="K26" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>134</v>
+      </c>
+      <c r="C27" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" t="s">
+        <v>136</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F27" t="s">
+        <v>140</v>
+      </c>
+      <c r="G27">
+        <v>348</v>
+      </c>
+      <c r="H27" t="s">
+        <v>141</v>
+      </c>
+      <c r="I27" t="s">
+        <v>41</v>
+      </c>
+      <c r="J27" t="s">
+        <v>138</v>
+      </c>
+      <c r="K27" t="s">
+        <v>137</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Link media images to Cloudflare R2, update audit data
Switch image src from local media_compressed to R2 bucket, update form-1/form-2 CSV data, primarydrains GeoJSON, audit status data and styles.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DA1C56-2AA9-4643-BD16-708DB569F739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185476C0-0041-45F2-8B60-7229C6AA1A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="143">
   <si>
     <t>area</t>
   </si>
@@ -446,6 +446,9 @@
   </si>
   <si>
     <t>V120</t>
+  </si>
+  <si>
+    <t>277</t>
   </si>
 </sst>
 </file>
@@ -594,7 +597,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -772,6 +775,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -935,13 +944,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1386,6 +1396,7 @@
       <c r="A3" t="s">
         <v>12</v>
       </c>
+      <c r="C3" s="4"/>
       <c r="D3" t="s">
         <v>13</v>
       </c>
@@ -1405,6 +1416,7 @@
       <c r="A4" t="s">
         <v>15</v>
       </c>
+      <c r="C4" s="4"/>
       <c r="D4" t="s">
         <v>13</v>
       </c>
@@ -1425,6 +1437,7 @@
       <c r="A5" t="s">
         <v>17</v>
       </c>
+      <c r="C5" s="4"/>
       <c r="D5" t="s">
         <v>18</v>
       </c>
@@ -1448,6 +1461,7 @@
       <c r="A6" t="s">
         <v>21</v>
       </c>
+      <c r="C6" s="4"/>
       <c r="D6" t="s">
         <v>18</v>
       </c>
@@ -1466,6 +1480,7 @@
       <c r="A7" t="s">
         <v>23</v>
       </c>
+      <c r="C7" s="4"/>
       <c r="D7" t="s">
         <v>24</v>
       </c>
@@ -1542,6 +1557,7 @@
       <c r="A10" t="s">
         <v>30</v>
       </c>
+      <c r="C10" s="4"/>
       <c r="D10" t="s">
         <v>31</v>
       </c>
@@ -1590,6 +1606,7 @@
       <c r="A12" t="s">
         <v>33</v>
       </c>
+      <c r="C12" s="4"/>
       <c r="D12" t="s">
         <v>34</v>
       </c>
@@ -1613,6 +1630,7 @@
       <c r="A13" t="s">
         <v>36</v>
       </c>
+      <c r="C13" s="4"/>
       <c r="E13" s="1"/>
       <c r="G13" s="1" t="s">
         <v>78</v>
@@ -1861,8 +1879,8 @@
       <c r="D22" t="s">
         <v>58</v>
       </c>
-      <c r="E22" s="1">
-        <v>269</v>
+      <c r="E22" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="F22" t="s">
         <v>59</v>
@@ -1879,6 +1897,7 @@
       <c r="A23" t="s">
         <v>60</v>
       </c>
+      <c r="C23" s="4"/>
       <c r="D23" t="s">
         <v>61</v>
       </c>

</xml_diff>

<commit_message>
Make filter dropdowns responsive at 1280px and 1024px breakpoints
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185476C0-0041-45F2-8B60-7229C6AA1A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366D4FC4-B84B-4BEA-BE78-A67F0893E595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="142">
   <si>
     <t>area</t>
   </si>
@@ -232,9 +232,6 @@
     <t>113,114,107</t>
   </si>
   <si>
-    <t>194,195</t>
-  </si>
-  <si>
     <t>241,253,255,250</t>
   </si>
   <si>
@@ -352,12 +349,6 @@
     <t>Ajay P, Aradhana J, Arjun P, Arshad, Cezanne Ali, Jagadeeswaran B, Jeesta Ghosh, Jenica Angelin, Jeya Shreya S, Malavika, Mayur Jeevan Das, Niharika Bedwal, Prakriti Mukherjee, Prakruti P C, R Swathi, Raghav Kumar, Ria Jagadev, Shradha Mishra, Soumili Santra, Sreeyuktha M V, Sudit Ilin, Tania Noble, Vaishnavi, Vishruti B</t>
   </si>
   <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t>90,274</t>
-  </si>
-  <si>
     <t>Aditya S</t>
   </si>
   <si>
@@ -449,6 +440,12 @@
   </si>
   <si>
     <t>277</t>
+  </si>
+  <si>
+    <t>89, 279, 278</t>
+  </si>
+  <si>
+    <t>194</t>
   </si>
 </sst>
 </file>
@@ -1327,7 +1324,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="10" max="10" width="57.28515625" customWidth="1"/>
@@ -1339,7 +1336,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1360,13 +1357,13 @@
         <v>6</v>
       </c>
       <c r="J1" t="s">
+        <v>93</v>
+      </c>
+      <c r="K1" t="s">
         <v>94</v>
       </c>
-      <c r="K1" t="s">
-        <v>95</v>
-      </c>
       <c r="L1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1383,7 +1380,7 @@
         <v>9</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
         <v>10</v>
@@ -1421,13 +1418,13 @@
         <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>
@@ -1448,7 +1445,7 @@
         <v>19</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H5" t="s">
         <v>20</v>
@@ -1491,7 +1488,7 @@
         <v>25</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H7" t="s">
         <v>26</v>
@@ -1505,7 +1502,7 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D8" t="s">
         <v>28</v>
@@ -1523,7 +1520,7 @@
         <v>28</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1531,16 +1528,16 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G9" s="1"/>
       <c r="I9" t="s">
@@ -1550,7 +1547,7 @@
         <v>31</v>
       </c>
       <c r="K9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1580,17 +1577,22 @@
         <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D11" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="1"/>
+      <c r="E11" s="1">
+        <v>267</v>
+      </c>
+      <c r="F11" t="s">
+        <v>35</v>
+      </c>
       <c r="G11" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I11" t="s">
         <v>41</v>
@@ -1599,7 +1601,7 @@
         <v>34</v>
       </c>
       <c r="K11" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1610,17 +1612,12 @@
       <c r="D12" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="1">
-        <v>267</v>
-      </c>
-      <c r="F12" t="s">
-        <v>35</v>
-      </c>
+      <c r="E12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H12" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I12" t="s">
         <v>11</v>
@@ -1633,7 +1630,7 @@
       <c r="C13" s="4"/>
       <c r="E13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H13" t="s">
         <v>37</v>
@@ -1647,7 +1644,7 @@
         <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
         <v>39</v>
@@ -1663,10 +1660,10 @@
         <v>41</v>
       </c>
       <c r="J14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1674,7 +1671,7 @@
         <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15" t="s">
         <v>39</v>
@@ -1690,10 +1687,10 @@
         <v>41</v>
       </c>
       <c r="J15" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1701,13 +1698,13 @@
         <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16" t="s">
         <v>39</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>70</v>
+        <v>141</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -1717,10 +1714,10 @@
         <v>41</v>
       </c>
       <c r="J16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1728,13 +1725,13 @@
         <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D17" t="s">
         <v>39</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F17" t="s">
         <v>46</v>
@@ -1744,10 +1741,10 @@
         <v>41</v>
       </c>
       <c r="J17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1755,13 +1752,13 @@
         <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
         <v>47</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F18" t="s">
         <v>46</v>
@@ -1774,7 +1771,7 @@
         <v>47</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1782,7 +1779,7 @@
         <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
         <v>49</v>
@@ -1798,13 +1795,13 @@
         <v>41</v>
       </c>
       <c r="J19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K19" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L19" t="s">
         <v>105</v>
-      </c>
-      <c r="L19" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1812,7 +1809,7 @@
         <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D20" t="s">
         <v>52</v>
@@ -1824,7 +1821,7 @@
         <v>54</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H20" t="s">
         <v>55</v>
@@ -1833,13 +1830,13 @@
         <v>41</v>
       </c>
       <c r="J20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1847,14 +1844,14 @@
         <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H21" t="s">
         <v>56</v>
@@ -1866,7 +1863,7 @@
         <v>8</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1874,13 +1871,13 @@
         <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D22" t="s">
         <v>58</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="F22" t="s">
         <v>59</v>
@@ -1908,7 +1905,7 @@
         <v>62</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H23" t="s">
         <v>63</v>
@@ -1919,108 +1916,90 @@
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" t="s">
+        <v>82</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" t="s">
         <v>84</v>
-      </c>
-      <c r="D24" t="s">
-        <v>83</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F24" t="s">
-        <v>85</v>
       </c>
       <c r="G24" s="1"/>
       <c r="I24" t="s">
         <v>41</v>
       </c>
       <c r="J24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="K24" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>84</v>
+        <v>124</v>
+      </c>
+      <c r="C25" t="s">
+        <v>126</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>111</v>
+        <v>125</v>
+      </c>
+      <c r="E25">
+        <v>276</v>
       </c>
       <c r="F25" t="s">
-        <v>85</v>
-      </c>
-      <c r="G25" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="H25" t="s">
+        <v>128</v>
+      </c>
       <c r="I25" t="s">
-        <v>11</v>
+        <v>41</v>
+      </c>
+      <c r="J25" t="s">
+        <v>129</v>
+      </c>
+      <c r="K25" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C26" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
-        <v>128</v>
-      </c>
-      <c r="E26">
-        <v>276</v>
+        <v>133</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="F26" t="s">
-        <v>43</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
+      </c>
+      <c r="G26">
+        <v>348</v>
       </c>
       <c r="H26" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="I26" t="s">
         <v>41</v>
       </c>
       <c r="J26" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="K26" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
         <v>134</v>
-      </c>
-      <c r="C27" t="s">
-        <v>135</v>
-      </c>
-      <c r="D27" t="s">
-        <v>136</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="F27" t="s">
-        <v>140</v>
-      </c>
-      <c r="G27">
-        <v>348</v>
-      </c>
-      <c r="H27" t="s">
-        <v>141</v>
-      </c>
-      <c r="I27" t="s">
-        <v>41</v>
-      </c>
-      <c r="J27" t="s">
-        <v>138</v>
-      </c>
-      <c r="K27" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consolidate geojson to root data/; fix responsive stats height
- Move all shared geojson layers to root data/json/ (primarydrains, secondarydrains, gba_boundary, gba_corporations, valley, and others)
- Update audit_dashboard/script.js paths from data/json/ to ../data/json/
- Remove per-dashboard copies of geojson from audit_dashboard/data/json/ and audit_status/data/json/
- Fix body.info-collapsed grid stats row staying 90px on 1280-1439px screens

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366D4FC4-B84B-4BEA-BE78-A67F0893E595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36ED6D0C-81EF-48AD-9CC1-349229AEFD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -941,7 +941,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -949,6 +949,10 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1497,56 +1501,56 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="5">
         <v>87</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="6" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="I9" t="s">
+      <c r="G9" s="5"/>
+      <c r="I9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="4" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1572,35 +1576,35 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="5">
         <v>267</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="4" t="s">
         <v>117</v>
       </c>
     </row>
@@ -1639,111 +1643,111 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="5">
         <v>270</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="I14" t="s">
+      <c r="G14" s="5"/>
+      <c r="I14" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="K14" s="6" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="5">
         <v>268</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="1"/>
-      <c r="I15" t="s">
+      <c r="G15" s="5"/>
+      <c r="I15" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="6" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="I16" t="s">
+      <c r="G16" s="5"/>
+      <c r="I16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="1"/>
-      <c r="I17" t="s">
+      <c r="G17" s="5"/>
+      <c r="I17" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" s="6" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1774,119 +1778,119 @@
         <v>108</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="5">
         <v>211</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="1"/>
-      <c r="I19" t="s">
+      <c r="G19" s="5"/>
+      <c r="I19" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L19" s="4" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="L20" t="s">
+      <c r="L20" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="G21" s="1" t="s">
+      <c r="E21" s="5"/>
+      <c r="G21" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="6" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G22" s="1"/>
-      <c r="I22" t="s">
+      <c r="G22" s="5"/>
+      <c r="I22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="4" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1914,27 +1918,27 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="1"/>
-      <c r="I24" t="s">
+      <c r="G24" s="5"/>
+      <c r="I24" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="K24" t="s">
+      <c r="K24" s="4" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2004,5 +2008,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update drains audit data, primarydrains geojson and add qmd source
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36ED6D0C-81EF-48AD-9CC1-349229AEFD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641140E5-F213-4E81-B4E1-E084118A432B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="149">
   <si>
     <t>area</t>
   </si>
@@ -446,6 +446,27 @@
   </si>
   <si>
     <t>194</t>
+  </si>
+  <si>
+    <t>Kengeri</t>
+  </si>
+  <si>
+    <t>Paani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RN181, </t>
+  </si>
+  <si>
+    <t>216,215</t>
+  </si>
+  <si>
+    <t>Paani Earth Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Madhuri, Richa </t>
+  </si>
+  <si>
+    <t>Abhayraj, Abhiraj, Akshat, Angelina, Anant, Ashwini, Deepa Chandrashekar, Gagana, Meenakshi, Radha B S, Rabi, Sethuraman, Snehit, Srinidhi, Sudarvizhi, Suneetha Nagaraj</t>
   </si>
 </sst>
 </file>
@@ -941,7 +962,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -953,6 +974,8 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1328,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="10" max="10" width="57.28515625" customWidth="1"/>
@@ -1918,27 +1941,27 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:12" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="5"/>
-      <c r="I24" s="4" t="s">
+      <c r="G24" s="8"/>
+      <c r="I24" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J24" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="K24" s="7" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2004,6 +2027,32 @@
       </c>
       <c r="K26" t="s">
         <v>134</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" t="s">
+        <v>143</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F27" t="s">
+        <v>144</v>
+      </c>
+      <c r="I27" t="s">
+        <v>41</v>
+      </c>
+      <c r="J27" t="s">
+        <v>147</v>
+      </c>
+      <c r="K27" t="s">
+        <v>148</v>
+      </c>
+      <c r="L27" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update audit status, download center, and story map assets
- Update audit_status README and drains_auditing data
- Replace typology.geojson with typology QMD analysis files
- Add geotiff aux.xml sidecar files for story map layers

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit_status/data/csv/drains_auditing.xlsx
+++ b/audit_status/data/csv/drains_auditing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\Decoding Stormwater Tools\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\01.DESIGN LAB\25-06_BSF SMALL GRANTS PROGRAMME\02_Implementation\04_Dashboard\02. Github Repo - DO NOT OPEN\mod-foundation\audit_status\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641140E5-F213-4E81-B4E1-E084118A432B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A4F2A7-9C1E-4591-B18C-B93A6A0F4871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5883F10E-228F-4B96-ADEB-DF7273A6A952}"/>
   </bookViews>
@@ -962,7 +962,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -975,7 +975,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1351,707 +1350,710 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F40D1B7E-5B77-4346-B197-6164F9686C92}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultColWidth="38.140625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="10" max="10" width="57.28515625" customWidth="1"/>
-    <col min="11" max="11" width="60" customWidth="1"/>
+    <col min="1" max="1" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" customWidth="1"/>
+    <col min="9" max="9" width="57.28515625" customWidth="1"/>
+    <col min="10" max="10" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>101</v>
+      </c>
       <c r="C1" t="s">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
       <c r="H1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I1" t="s">
-        <v>6</v>
+        <v>93</v>
       </c>
       <c r="J1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K1" t="s">
-        <v>94</v>
-      </c>
-      <c r="L1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
       <c r="H2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F3" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="I3" t="s">
+      <c r="F3" s="1"/>
+      <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I4" t="s">
+      <c r="H4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>75</v>
       </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
       <c r="H5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E6" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="I6" t="s">
+      <c r="F6" s="1"/>
+      <c r="H6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F7" t="s">
+      <c r="E7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>76</v>
       </c>
+      <c r="G7" t="s">
+        <v>26</v>
+      </c>
       <c r="H7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
+      <c r="B8" s="4" t="s">
+        <v>119</v>
+      </c>
       <c r="C8" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="5">
+      <c r="D8" s="5">
         <v>87</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>29</v>
       </c>
+      <c r="H8" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>30</v>
       </c>
+      <c r="B9" s="4" t="s">
+        <v>121</v>
+      </c>
       <c r="C9" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="D9" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="E9" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F9" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="H9" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I9" s="4" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K9" s="4" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F10" t="s">
+      <c r="E10" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="H10" t="s">
+        <v>11</v>
+      </c>
       <c r="I10" t="s">
-        <v>11</v>
-      </c>
-      <c r="J10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
+      <c r="B11" s="4" t="s">
+        <v>120</v>
+      </c>
       <c r="C11" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="5">
+      <c r="D11" s="5">
         <v>267</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>113</v>
       </c>
+      <c r="G11" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="H11" s="4" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K11" s="4" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="G12" s="1" t="s">
+      <c r="D12" s="1"/>
+      <c r="F12" s="1" t="s">
         <v>114</v>
       </c>
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
       <c r="H12" t="s">
-        <v>112</v>
-      </c>
-      <c r="I12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="E13" s="1"/>
-      <c r="G13" s="1" t="s">
+      <c r="B13" s="4"/>
+      <c r="D13" s="1"/>
+      <c r="F13" s="1" t="s">
         <v>77</v>
       </c>
+      <c r="G13" t="s">
+        <v>37</v>
+      </c>
       <c r="H13" t="s">
-        <v>37</v>
-      </c>
-      <c r="I13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>38</v>
       </c>
+      <c r="B14" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="C14" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="5">
+      <c r="D14" s="5">
         <v>270</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="H14" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I14" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J14" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K14" s="6" t="s">
+      <c r="J14" s="6" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="B15" s="4" t="s">
+        <v>85</v>
+      </c>
       <c r="C15" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="5">
+      <c r="D15" s="5">
         <v>268</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="H15" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I15" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J15" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="J15" s="6" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>44</v>
       </c>
+      <c r="B16" s="4" t="s">
+        <v>86</v>
+      </c>
       <c r="C16" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="H16" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I16" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J16" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K16" s="6" t="s">
+      <c r="J16" s="6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>45</v>
       </c>
+      <c r="B17" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="C17" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="H17" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J17" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="J17" s="6" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
       <c r="C18" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F18" t="s">
+      <c r="E18" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="H18" t="s">
+        <v>41</v>
+      </c>
       <c r="I18" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" t="s">
         <v>47</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>48</v>
       </c>
+      <c r="B19" s="4" t="s">
+        <v>90</v>
+      </c>
       <c r="C19" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="5">
+      <c r="D19" s="5">
         <v>211</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="H19" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I19" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J19" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="K19" s="6" t="s">
+      <c r="J19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>
+      <c r="B20" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="C20" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="E20" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>78</v>
       </c>
+      <c r="G20" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="H20" s="4" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J20" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="J20" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="L20" s="4" t="s">
+      <c r="K20" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="B21" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="C21" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="G21" s="5" t="s">
+      <c r="D21" s="5"/>
+      <c r="F21" s="5" t="s">
         <v>71</v>
       </c>
+      <c r="G21" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="H21" s="4" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="J21" s="6" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>57</v>
       </c>
+      <c r="B22" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="C22" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="H22" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="I22" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J22" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="4"/>
-      <c r="D23" t="s">
+      <c r="B23" s="4"/>
+      <c r="C23" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="1">
+      <c r="D23" s="1">
         <v>40</v>
       </c>
-      <c r="F23" t="s">
+      <c r="E23" t="s">
         <v>62</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>79</v>
       </c>
+      <c r="G23" t="s">
+        <v>63</v>
+      </c>
       <c r="H23" t="s">
-        <v>63</v>
-      </c>
-      <c r="I23" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="C24" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="D24" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="E24" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="8"/>
-      <c r="I24" s="7" t="s">
+      <c r="F24" s="1"/>
+      <c r="H24" t="s">
         <v>41</v>
       </c>
-      <c r="J24" s="7" t="s">
+      <c r="I24" t="s">
         <v>109</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="J24" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>124</v>
       </c>
+      <c r="B25" t="s">
+        <v>126</v>
+      </c>
       <c r="C25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D25" t="s">
         <v>125</v>
       </c>
-      <c r="E25">
+      <c r="D25">
         <v>276</v>
       </c>
-      <c r="F25" t="s">
+      <c r="E25" t="s">
         <v>43</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>127</v>
       </c>
+      <c r="G25" t="s">
+        <v>128</v>
+      </c>
       <c r="H25" t="s">
-        <v>128</v>
+        <v>41</v>
       </c>
       <c r="I25" t="s">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="J25" t="s">
-        <v>129</v>
-      </c>
-      <c r="K25" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>131</v>
       </c>
+      <c r="B26" t="s">
+        <v>132</v>
+      </c>
       <c r="C26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" t="s">
         <v>133</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F26" t="s">
+      <c r="E26" t="s">
         <v>137</v>
       </c>
-      <c r="G26">
+      <c r="F26">
         <v>348</v>
       </c>
+      <c r="G26" t="s">
+        <v>138</v>
+      </c>
       <c r="H26" t="s">
-        <v>138</v>
+        <v>41</v>
       </c>
       <c r="I26" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="J26" t="s">
-        <v>135</v>
-      </c>
-      <c r="K26" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>142</v>
       </c>
-      <c r="D27" t="s">
+      <c r="C27" t="s">
         <v>143</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F27" t="s">
+      <c r="E27" t="s">
         <v>144</v>
       </c>
+      <c r="H27" t="s">
+        <v>41</v>
+      </c>
       <c r="I27" t="s">
-        <v>41</v>
+        <v>147</v>
       </c>
       <c r="J27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K27" t="s">
-        <v>148</v>
-      </c>
-      <c r="L27" t="s">
         <v>146</v>
       </c>
     </row>

</xml_diff>